<commit_message>
Reporte proceso de cinemática y resultados
</commit_message>
<xml_diff>
--- a/datos/tabla_DH/Robot_Resumen.xlsx
+++ b/datos/tabla_DH/Robot_Resumen.xlsx
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="17" uniqueCount="15">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="17" uniqueCount="14">
   <si>
     <t xml:space="preserve">N</t>
   </si>
@@ -62,9 +62,6 @@
   </si>
   <si>
     <t xml:space="preserve">r</t>
-  </si>
-  <si>
-    <t xml:space="preserve">p</t>
   </si>
 </sst>
 </file>
@@ -146,20 +143,24 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="5">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -355,228 +356,228 @@
   <dimension ref="A1:M6"/>
   <sheetFormatPr defaultColWidth="10.54296875" defaultRowHeight="14.25" customHeight="true" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="2.33"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="5.33"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="4"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="4" style="0" width="5.44"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="0" width="4.48"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="0" width="6.44"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="0" width="7.44"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="10" min="9" style="0" width="8.44"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="11" min="11" style="0" width="8"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="12" min="12" style="0" width="8.34"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="2.33"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="5.33"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="1" width="4"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="4" style="1" width="5.44"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="1" width="4.48"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="1" width="6.44"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="1" width="7.44"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="10" min="9" style="1" width="8.44"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="11" min="11" style="1" width="8"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="12" min="12" style="1" width="8.34"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1" s="0" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="1" t="s">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="2" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="0" t="s">
+      <c r="C1" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="0" t="s">
+      <c r="D1" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="0" t="s">
+      <c r="E1" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="0" t="s">
+      <c r="F1" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="G1" s="0" t="s">
+      <c r="G1" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="H1" s="0" t="s">
+      <c r="H1" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="I1" s="0" t="s">
+      <c r="I1" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="J1" s="0" t="s">
+      <c r="J1" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="K1" s="0" t="s">
+      <c r="K1" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="L1" s="0" t="s">
+      <c r="L1" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="M1" s="0" t="s">
+      <c r="M1" s="1" t="s">
         <v>12</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2" s="0" t="n">
+      <c r="A2" s="1" t="n">
         <v>1</v>
       </c>
-      <c r="B2" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="C2" s="2" t="n">
-        <v>7</v>
-      </c>
-      <c r="D2" s="2" t="n">
-        <v>3</v>
-      </c>
-      <c r="E2" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="F2" s="2" t="s">
+      <c r="B2" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C2" s="3" t="n">
+        <v>50</v>
+      </c>
+      <c r="D2" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="E2" s="3" t="n">
+        <v>-90</v>
+      </c>
+      <c r="F2" s="3" t="s">
         <v>13</v>
       </c>
-      <c r="G2" s="2" t="n">
-        <v>-90</v>
-      </c>
-      <c r="H2" s="2" t="n">
-        <v>90</v>
-      </c>
-      <c r="I2" s="2" t="n">
+      <c r="G2" s="3" t="n">
+        <v>-180</v>
+      </c>
+      <c r="H2" s="3" t="n">
         <v>180</v>
       </c>
-      <c r="J2" s="2" t="n">
+      <c r="I2" s="3" t="n">
+        <v>180</v>
+      </c>
+      <c r="J2" s="3" t="n">
         <v>360</v>
       </c>
-      <c r="K2" s="2" t="n">
-        <v>8</v>
-      </c>
-      <c r="L2" s="2" t="n">
+      <c r="K2" s="3" t="n">
+        <v>134</v>
+      </c>
+      <c r="L2" s="3" t="n">
         <v>0.1</v>
       </c>
-      <c r="M2" s="2" t="n">
+      <c r="M2" s="3" t="n">
         <v>0.2</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A3" s="0" t="n">
+      <c r="A3" s="1" t="n">
         <f aca="false">A2+1</f>
         <v>2</v>
       </c>
-      <c r="B3" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="C3" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="D3" s="2" t="n">
-        <v>3</v>
-      </c>
-      <c r="E3" s="2" t="n">
+      <c r="B3" s="3" t="n">
+        <v>90</v>
+      </c>
+      <c r="C3" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="D3" s="3" t="n">
+        <v>50</v>
+      </c>
+      <c r="E3" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="F3" s="3" t="s">
+        <v>13</v>
+      </c>
+      <c r="G3" s="3" t="n">
         <v>-90</v>
       </c>
-      <c r="F3" s="2" t="s">
-        <v>13</v>
-      </c>
-      <c r="G3" s="2" t="n">
-        <v>-90</v>
-      </c>
-      <c r="H3" s="2" t="n">
+      <c r="H3" s="3" t="n">
         <v>90</v>
       </c>
-      <c r="I3" s="2" t="n">
+      <c r="I3" s="3" t="n">
         <v>180</v>
       </c>
-      <c r="J3" s="2" t="n">
+      <c r="J3" s="3" t="n">
         <v>360</v>
       </c>
-      <c r="K3" s="2" t="n">
-        <v>50</v>
-      </c>
-      <c r="L3" s="2" t="n">
+      <c r="K3" s="3" t="n">
+        <v>110</v>
+      </c>
+      <c r="L3" s="3" t="n">
         <v>0.1</v>
       </c>
-      <c r="M3" s="2" t="n">
+      <c r="M3" s="3" t="n">
         <v>0.2</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A4" s="0" t="n">
+      <c r="A4" s="1" t="n">
         <f aca="false">A3+1</f>
         <v>3</v>
       </c>
-      <c r="B4" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="C4" s="2" t="n">
-        <v>2</v>
-      </c>
-      <c r="D4" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="E4" s="2" t="n">
+      <c r="B4" s="3" t="n">
         <v>-90</v>
       </c>
-      <c r="F4" s="2" t="s">
+      <c r="C4" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="D4" s="3" t="n">
+        <v>43</v>
+      </c>
+      <c r="E4" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="F4" s="3" t="s">
         <v>13</v>
       </c>
-      <c r="G4" s="2" t="n">
+      <c r="G4" s="3" t="n">
         <v>-90</v>
       </c>
-      <c r="H4" s="2" t="n">
+      <c r="H4" s="3" t="n">
         <v>90</v>
       </c>
-      <c r="I4" s="2" t="n">
+      <c r="I4" s="3" t="n">
         <v>180</v>
       </c>
-      <c r="J4" s="2" t="n">
+      <c r="J4" s="3" t="n">
         <v>360</v>
       </c>
-      <c r="K4" s="2" t="n">
-        <v>30</v>
-      </c>
-      <c r="L4" s="2" t="n">
+      <c r="K4" s="3" t="n">
+        <v>50</v>
+      </c>
+      <c r="L4" s="3" t="n">
         <v>0.1</v>
       </c>
-      <c r="M4" s="2" t="n">
+      <c r="M4" s="3" t="n">
         <v>0.2</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="0" t="n">
+      <c r="A5" s="1" t="n">
         <f aca="false">A4+1</f>
         <v>4</v>
       </c>
-      <c r="B5" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="C5" s="2" t="n">
-        <v>5</v>
-      </c>
-      <c r="D5" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="E5" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="F5" s="2" t="s">
-        <v>14</v>
-      </c>
-      <c r="G5" s="2" t="n">
-        <v>3</v>
-      </c>
-      <c r="H5" s="2" t="n">
-        <v>7</v>
-      </c>
-      <c r="I5" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="J5" s="2" t="n">
-        <v>2</v>
-      </c>
-      <c r="K5" s="2" t="n">
-        <v>10</v>
-      </c>
-      <c r="L5" s="2" t="n">
+      <c r="B5" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C5" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="D5" s="3" t="n">
+        <v>6</v>
+      </c>
+      <c r="E5" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="F5" s="3" t="s">
+        <v>13</v>
+      </c>
+      <c r="G5" s="3" t="n">
+        <v>-90</v>
+      </c>
+      <c r="H5" s="3" t="n">
+        <v>90</v>
+      </c>
+      <c r="I5" s="3" t="n">
+        <v>180</v>
+      </c>
+      <c r="J5" s="3" t="n">
+        <v>360</v>
+      </c>
+      <c r="K5" s="3" t="n">
+        <v>19</v>
+      </c>
+      <c r="L5" s="3" t="n">
         <v>0.1</v>
       </c>
-      <c r="M5" s="2" t="n">
+      <c r="M5" s="3" t="n">
         <v>0.2</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H6" s="3"/>
+      <c r="H6" s="4"/>
     </row>
   </sheetData>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>

</xml_diff>